<commit_message>
MACD scan results 2026-10-06
</commit_message>
<xml_diff>
--- a/results/macd_2026-10-06.xlsx
+++ b/results/macd_2026-10-06.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E78"/>
+  <dimension ref="A1:E79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,25 +444,21 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>ECHO</t>
-        </is>
-      </c>
+      <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
+          <t>AAL</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>AAOI</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>ABSI</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ALAB</t>
+          <t>ABSI</t>
         </is>
       </c>
     </row>
@@ -475,13 +471,13 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ACLS</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>AMRX</t>
+          <t>ACLS</t>
         </is>
       </c>
     </row>
@@ -494,13 +490,13 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>ARW</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ANGO</t>
+          <t>ALAB</t>
         </is>
       </c>
     </row>
@@ -508,18 +504,18 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>ASTS</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AEHR</t>
+          <t>AVPT</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>AMAT</t>
         </is>
       </c>
     </row>
@@ -527,18 +523,18 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>COST</t>
+          <t>ATMU</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AMAT</t>
+          <t>AVT</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BGC</t>
+          <t>AMD</t>
         </is>
       </c>
     </row>
@@ -546,18 +542,18 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>EVRG</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ARW</t>
+          <t>AXTI</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CHEF</t>
+          <t>APA</t>
         </is>
       </c>
     </row>
@@ -565,18 +561,18 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>FHB</t>
+          <t>CEG</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>BELFB</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>ARM</t>
         </is>
       </c>
     </row>
@@ -584,18 +580,18 @@
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>HON</t>
+          <t>COST</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AVPT</t>
+          <t>CECO</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>ASML</t>
         </is>
       </c>
     </row>
@@ -603,18 +599,18 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>IBOC</t>
+          <t>EVRG</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AVT</t>
+          <t>CGNX</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>CVCO</t>
+          <t>BGC</t>
         </is>
       </c>
     </row>
@@ -622,18 +618,18 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>IDXX</t>
+          <t>FELE</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AXTI</t>
+          <t>CLOV</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>CAKE</t>
         </is>
       </c>
     </row>
@@ -641,18 +637,18 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>LIN</t>
+          <t>FHB</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>CAKE</t>
+          <t>COHR</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>COHU</t>
         </is>
       </c>
     </row>
@@ -660,18 +656,18 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>MKSI</t>
+          <t>GPGI</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CAMT</t>
+          <t>COKE</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>FORM</t>
+          <t>DDOG</t>
         </is>
       </c>
     </row>
@@ -679,18 +675,18 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>MYRG</t>
+          <t>HON</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CDNA</t>
+          <t>CORT</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>ILMN</t>
+          <t>FORM</t>
         </is>
       </c>
     </row>
@@ -698,18 +694,18 @@
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>NTES</t>
+          <t>IDXX</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>CGNX</t>
+          <t>CR</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>IOVA</t>
+          <t>IBRX</t>
         </is>
       </c>
     </row>
@@ -717,18 +713,18 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>NVTS</t>
+          <t>LPTH</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>COHR</t>
+          <t>CRDO</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>IRDM</t>
+          <t>ICHR</t>
         </is>
       </c>
     </row>
@@ -736,18 +732,18 @@
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
-          <t>PECO</t>
+          <t>LSTR</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>COHU</t>
+          <t>CRWD</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>KOD</t>
+          <t>KLAC</t>
         </is>
       </c>
     </row>
@@ -755,18 +751,18 @@
       <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr">
         <is>
-          <t>POET</t>
+          <t>LWLG</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>CORT</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>LGND</t>
+          <t>KLIC</t>
         </is>
       </c>
     </row>
@@ -774,18 +770,18 @@
       <c r="A19" t="inlineStr"/>
       <c r="B19" t="inlineStr">
         <is>
-          <t>POWL</t>
+          <t>MYRG</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>CR</t>
+          <t>CVCO</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>LILAK</t>
+          <t>KOD</t>
         </is>
       </c>
     </row>
@@ -793,18 +789,18 @@
       <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr">
         <is>
-          <t>PWP</t>
+          <t>ORLY</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>CRAI</t>
+          <t>CVLT</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>LAUR</t>
         </is>
       </c>
     </row>
@@ -812,18 +808,18 @@
       <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr">
         <is>
-          <t>RYAAY</t>
+          <t>OSW</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>CVLT</t>
+          <t>DIOD</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>MEDP</t>
+          <t>LRCX</t>
         </is>
       </c>
     </row>
@@ -831,18 +827,18 @@
       <c r="A22" t="inlineStr"/>
       <c r="B22" t="inlineStr">
         <is>
-          <t>STRL</t>
+          <t>PECO</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>CYRX</t>
+          <t>ENTG</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>MEOH</t>
         </is>
       </c>
     </row>
@@ -850,48 +846,56 @@
       <c r="A23" t="inlineStr"/>
       <c r="B23" t="inlineStr">
         <is>
-          <t>SUPN</t>
+          <t>POET</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>DIOD</t>
+          <t>FAST</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>MRX</t>
+          <t>NNBR</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr"/>
-      <c r="B24" t="inlineStr"/>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>RYAAY</t>
+        </is>
+      </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ENTG</t>
+          <t>FFIV</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>PAYO</t>
+          <t>ONC</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
-      <c r="B25" t="inlineStr"/>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>TCBI</t>
+        </is>
+      </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>FAST</t>
+          <t>FLEX</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>QMCO</t>
+          <t>PAYO</t>
         </is>
       </c>
     </row>
@@ -900,13 +904,13 @@
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>FFIV</t>
+          <t>FOSL</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SBLK</t>
+          <t>PDFS</t>
         </is>
       </c>
     </row>
@@ -915,13 +919,13 @@
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>FLEX</t>
+          <t>FRHC</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>SHOO</t>
+          <t>PLPC</t>
         </is>
       </c>
     </row>
@@ -930,13 +934,13 @@
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>FOSL</t>
+          <t>FROG</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SIMO</t>
+          <t>PLXS</t>
         </is>
       </c>
     </row>
@@ -945,13 +949,13 @@
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>FRHC</t>
+          <t>FTNT</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>SMTC</t>
+          <t>RXT</t>
         </is>
       </c>
     </row>
@@ -960,13 +964,13 @@
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>FROG</t>
+          <t>GCT</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>VICR</t>
+          <t>SANM</t>
         </is>
       </c>
     </row>
@@ -975,13 +979,13 @@
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>FTNT</t>
+          <t>GMAB</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>VSXY</t>
+          <t>SHIP</t>
         </is>
       </c>
     </row>
@@ -990,13 +994,13 @@
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>GH</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>XMTR</t>
+          <t>SHOO</t>
         </is>
       </c>
     </row>
@@ -1005,13 +1009,13 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>GRAL</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>XNCR</t>
+          <t>SLAB</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1028,11 @@
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>STLN</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr"/>
@@ -1035,47 +1043,63 @@
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>TER</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr"/>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>IBRX</t>
+          <t>IDCC</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>TRMD</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr"/>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ICHR</t>
+          <t>IESC</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>VSXY</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>IDCC</t>
+          <t>IRDM</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>XNCR</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr"/>
       <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
-          <t>IESC</t>
+          <t>KOPN</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1086,7 +1110,7 @@
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>KLAC</t>
+          <t>LECO</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -1097,7 +1121,7 @@
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
-          <t>KLIC</t>
+          <t>LFUS</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -1108,7 +1132,7 @@
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>LAUR</t>
+          <t>LILAK</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -1119,7 +1143,7 @@
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
-          <t>LECO</t>
+          <t>LIND</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -1130,7 +1154,7 @@
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
-          <t>LFUS</t>
+          <t>LITE</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -1141,7 +1165,7 @@
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
-          <t>LIND</t>
+          <t>LOGI</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -1152,7 +1176,7 @@
       <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
-          <t>LITE</t>
+          <t>LSCC</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
@@ -1163,7 +1187,7 @@
       <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>MAR</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
@@ -1174,7 +1198,7 @@
       <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
-          <t>LSCC</t>
+          <t>MPWR</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
@@ -1185,7 +1209,7 @@
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
-          <t>MPWR</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
@@ -1196,7 +1220,7 @@
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>MRX</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
@@ -1207,7 +1231,7 @@
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr">
         <is>
-          <t>MTSI</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
@@ -1218,7 +1242,7 @@
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr">
         <is>
-          <t>MXL</t>
+          <t>MTSI</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
@@ -1229,7 +1253,7 @@
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr">
         <is>
-          <t>NDSN</t>
+          <t>MXL</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
@@ -1240,7 +1264,7 @@
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr">
         <is>
-          <t>NNBR</t>
+          <t>NDSN</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
@@ -1251,7 +1275,7 @@
       <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr">
         <is>
-          <t>NTAP</t>
+          <t>NOVT</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
@@ -1262,7 +1286,7 @@
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr">
         <is>
-          <t>NTNX</t>
+          <t>NTAP</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
@@ -1273,7 +1297,7 @@
       <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>NTCT</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
@@ -1284,7 +1308,7 @@
       <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr">
         <is>
-          <t>OKTA</t>
+          <t>NTNX</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
@@ -1295,7 +1319,7 @@
       <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
-          <t>OUST</t>
+          <t>NUTX</t>
         </is>
       </c>
       <c r="D59" t="inlineStr"/>
@@ -1306,7 +1330,7 @@
       <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="D60" t="inlineStr"/>
@@ -1317,7 +1341,7 @@
       <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>OKTA</t>
         </is>
       </c>
       <c r="D61" t="inlineStr"/>
@@ -1328,7 +1352,7 @@
       <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr">
         <is>
-          <t>PAYS</t>
+          <t>OPTX</t>
         </is>
       </c>
       <c r="D62" t="inlineStr"/>
@@ -1339,7 +1363,7 @@
       <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr">
         <is>
-          <t>PCVX</t>
+          <t>OUST</t>
         </is>
       </c>
       <c r="D63" t="inlineStr"/>
@@ -1350,7 +1374,7 @@
       <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr">
         <is>
-          <t>PENG</t>
+          <t>P</t>
         </is>
       </c>
       <c r="D64" t="inlineStr"/>
@@ -1361,7 +1385,7 @@
       <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="D65" t="inlineStr"/>
@@ -1372,7 +1396,7 @@
       <c r="B66" t="inlineStr"/>
       <c r="C66" t="inlineStr">
         <is>
-          <t>PLXS</t>
+          <t>PCVX</t>
         </is>
       </c>
       <c r="D66" t="inlineStr"/>
@@ -1383,7 +1407,7 @@
       <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr">
         <is>
-          <t>PRCH</t>
+          <t>PENG</t>
         </is>
       </c>
       <c r="D67" t="inlineStr"/>
@@ -1394,7 +1418,7 @@
       <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr">
         <is>
-          <t>QLYS</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="D68" t="inlineStr"/>
@@ -1405,7 +1429,7 @@
       <c r="B69" t="inlineStr"/>
       <c r="C69" t="inlineStr">
         <is>
-          <t>RVMD</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="D69" t="inlineStr"/>
@@ -1416,7 +1440,7 @@
       <c r="B70" t="inlineStr"/>
       <c r="C70" t="inlineStr">
         <is>
-          <t>SANM</t>
+          <t>PRCH</t>
         </is>
       </c>
       <c r="D70" t="inlineStr"/>
@@ -1427,7 +1451,7 @@
       <c r="B71" t="inlineStr"/>
       <c r="C71" t="inlineStr">
         <is>
-          <t>SCSC</t>
+          <t>QLYS</t>
         </is>
       </c>
       <c r="D71" t="inlineStr"/>
@@ -1438,7 +1462,7 @@
       <c r="B72" t="inlineStr"/>
       <c r="C72" t="inlineStr">
         <is>
-          <t>SHOP</t>
+          <t>QMCO</t>
         </is>
       </c>
       <c r="D72" t="inlineStr"/>
@@ -1449,7 +1473,7 @@
       <c r="B73" t="inlineStr"/>
       <c r="C73" t="inlineStr">
         <is>
-          <t>SITM</t>
+          <t>SHOP</t>
         </is>
       </c>
       <c r="D73" t="inlineStr"/>
@@ -1460,7 +1484,7 @@
       <c r="B74" t="inlineStr"/>
       <c r="C74" t="inlineStr">
         <is>
-          <t>SLAB</t>
+          <t>SIMO</t>
         </is>
       </c>
       <c r="D74" t="inlineStr"/>
@@ -1471,7 +1495,7 @@
       <c r="B75" t="inlineStr"/>
       <c r="C75" t="inlineStr">
         <is>
-          <t>SYNA</t>
+          <t>SITM</t>
         </is>
       </c>
       <c r="D75" t="inlineStr"/>
@@ -1482,7 +1506,7 @@
       <c r="B76" t="inlineStr"/>
       <c r="C76" t="inlineStr">
         <is>
-          <t>TER</t>
+          <t>SMTC</t>
         </is>
       </c>
       <c r="D76" t="inlineStr"/>
@@ -1493,7 +1517,7 @@
       <c r="B77" t="inlineStr"/>
       <c r="C77" t="inlineStr">
         <is>
-          <t>TRMD</t>
+          <t>SYNA</t>
         </is>
       </c>
       <c r="D77" t="inlineStr"/>
@@ -1510,6 +1534,17 @@
       <c r="D78" t="inlineStr"/>
       <c r="E78" t="inlineStr"/>
     </row>
+    <row r="79">
+      <c r="A79" t="inlineStr"/>
+      <c r="B79" t="inlineStr"/>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>XMTR</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>